<commit_message>
Arbeitspaket change + Funktionen plan
</commit_message>
<xml_diff>
--- a/doc/Abgaben/BMSD24a-Finanzappli-Arbeitspakete.xlsx
+++ b/doc/Abgaben/BMSD24a-Finanzappli-Arbeitspakete.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\poles\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\poles\Desktop\Finanzappli\doc\Abgaben\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68ADA497-81DD-4B96-AA1D-62328CF72638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAC9BC36-AFB4-4025-ACEB-9868F1F056AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1981,7 +1981,7 @@
         <v>99</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>18</v>
+        <v>93</v>
       </c>
       <c r="F10" s="12" t="s">
         <v>19</v>
@@ -7346,7 +7346,7 @@
       </c>
       <c r="C8" s="48" t="str">
         <f>IF($A8="","",VLOOKUP($A8,Arbeitspakete!$A$3:$M$999,C$2,FALSE))</f>
-        <v>Offen</v>
+        <v>FERTIG</v>
       </c>
       <c r="D8" s="67">
         <f>IF($A8="","",VLOOKUP($A8,Arbeitspakete!$A$3:$M$999,D$2,FALSE))</f>
@@ -12297,6 +12297,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="7428d6b1-3919-45ca-a810-a9f24c98c389" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100474F511FE9344346B3B565D439640D46" ma:contentTypeVersion="12" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="21da785c10f7c5f43f37cca8904c7fb7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="7428d6b1-3919-45ca-a810-a9f24c98c389" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="602e5a62d6284efa4700467c044525af" ns3:_="">
     <xsd:import namespace="7428d6b1-3919-45ca-a810-a9f24c98c389"/>
@@ -12490,37 +12507,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="7428d6b1-3919-45ca-a810-a9f24c98c389" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1C6C3F3-F3AC-4155-B379-CB7CE3B9DB83}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4701EF02-EC87-4C82-B449-CF5094A99EE7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="7428d6b1-3919-45ca-a810-a9f24c98c389"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -12542,9 +12532,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4701EF02-EC87-4C82-B449-CF5094A99EE7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1C6C3F3-F3AC-4155-B379-CB7CE3B9DB83}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="7428d6b1-3919-45ca-a810-a9f24c98c389"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>